<commit_message>
v2: real formulas, correct Dubai transport/PDI constants
</commit_message>
<xml_diff>
--- a/Pricing_Sheet_Template.xlsx
+++ b/Pricing_Sheet_Template.xlsx
@@ -16,8 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="7">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,13 +45,18 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="000000FF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -58,7 +65,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +75,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -151,20 +163,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -530,15 +553,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -565,7 +589,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>COST BUILD-UP (per unit)</t>
+          <t>CONSTANTS / INPUTS</t>
         </is>
       </c>
       <c r="B5" s="4" t="n"/>
@@ -574,235 +598,339 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>SAR</t>
-        </is>
+          <t>FX Rate (USD → SAR)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>3.75</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Ex-works Price</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>{{ExWorksUSD}}</t>
-        </is>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Customs Duty %</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Non-witness Test Charge</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>{{TestChargeUSD}}</t>
-        </is>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Master Freight Rate (Italy only, % of ex-works)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>0.14</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Ex-works Cost Basis (USD)</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Transport per truck, Dubai (SAR)</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Other Customs Clearance, Dubai (SAR)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Qty per Truck (Dubai)</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>{{QtyPerTruck}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>PDI (SAR)</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>{{PDISAR}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Is Italy Origin? (1=Yes, 0=No)</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>{{IsItalyOriginFlag}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Ex-works Price (USD)</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>{{ExWorksTotalUSD}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Customs Duty (15%)</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>{{DutyUSD}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Freight (Italy: 14% of ex-works | Dubai: fixed per truck)</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>{{FreightUSD}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Landed Cost (SAR, after FX 3.75)</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>{{LandedCostSAR}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>PDI &amp; Transport (SAR)</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>{{PDISAR}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>ACTUAL COST per Unit (SAR)</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>{{ActualCostSAR}}</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>COST BUILD-UP</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>SAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Freight Cost (Italy: 14% of ex-works | Dubai: 0, uses truck transport below)</t>
+        </is>
+      </c>
+      <c r="B18" s="13">
+        <f>IF(B13=1,B14*B8,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Custom Duty</t>
+        </is>
+      </c>
+      <c r="B19" s="13">
+        <f>B14*B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Total (USD)</t>
+        </is>
+      </c>
+      <c r="B20" s="15">
+        <f>B14+B18+B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Est. Landed Cost (SAR)</t>
+        </is>
+      </c>
+      <c r="C21" s="15">
+        <f>B20*B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Dubai Transport + Clearance (SAR, per truck) — n/a for Italy</t>
+        </is>
+      </c>
+      <c r="C22" s="13">
+        <f>IF(B13=1,0,B9+B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Transport Cost per Unit (SAR)</t>
+        </is>
+      </c>
+      <c r="C23" s="13">
+        <f>IF(B13=1,0,C22/B11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Landed Cost per Unit (SAR)</t>
+        </is>
+      </c>
+      <c r="C24" s="15">
+        <f>C21+C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>Total Landed Cost per Unit (SAR)</t>
+        </is>
+      </c>
+      <c r="C25" s="17">
+        <f>C24+B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
           <t>PRICING TIERS</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="5" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Margin</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>Unit Price (SAR)</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Unit Profit (SAR)</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E28" s="12" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Total Price (SAR)</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>Total Profit (SAR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Opening Price</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>13.0%</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>{{OpeningPriceUnit}}</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>{{OpeningProfitUnit}}</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="B29" s="18" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="C29" s="19">
+        <f>C25/(1-B29)</f>
+        <v/>
+      </c>
+      <c r="D29" s="19">
+        <f>C29-C25</f>
+        <v/>
+      </c>
+      <c r="E29" s="20" t="inlineStr">
         <is>
           <t>{{Quantity}}</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>{{OpeningPriceTotal}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Floor / Final Price</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>10.0%</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>{{FloorPriceUnit}}</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>{{FloorProfitUnit}}</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="F29" s="19">
+        <f>C29*E29</f>
+        <v/>
+      </c>
+      <c r="G29" s="19">
+        <f>D29*E29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Final / Floor Price</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C30" s="19">
+        <f>C25/(1-B30)</f>
+        <v/>
+      </c>
+      <c r="D30" s="19">
+        <f>C30-C25</f>
+        <v/>
+      </c>
+      <c r="E30" s="20" t="inlineStr">
         <is>
           <t>{{Quantity}}</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>{{FloorPriceTotal}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>Note: Customer-facing quotation shows Opening Price only. Floor price is internal negotiation fallback — not to be disclosed to customer.</t>
+      <c r="F30" s="19">
+        <f>C30*E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="19">
+        <f>D30*E30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>Note: Customer-facing quotation shows Opening Price only. Floor/Final price is internal negotiation fallback — not disclosed to customer. All cells above (except yellow inputs) are live formulas — safe to review and audit.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>